<commit_message>
NTI Workflow v0.3: detaljepanel, zoom, import-advarsler og oprydning.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/samples/sample-lifecycle.xlsx
+++ b/samples/sample-lifecycle.xlsx
@@ -651,7 +651,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Engineer:Read:Allow;Write:Allow;Delete:Deny;Download:Allow;Manager:Read:Allow;Write:Allow;Delete:Allow;Download:Allow</t>
+          <t>Engineer: Read: Allow, Write: Allow, Delete: Deny, Download: Allow; Manager: Read: Allow, Write: Allow, Delete: Allow, Download: Allow</t>
         </is>
       </c>
     </row>
@@ -673,7 +673,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Engineer:Read:Allow;Write:Deny;Delete:Deny;Download:Allow;Manager:Read:Allow;Write:Allow;Delete:Allow;Download:Allow</t>
+          <t>Engineer: Read: Allow, Write: Deny, Delete: Deny, Download: Allow; Manager: Read: Allow, Write: Allow, Delete: Allow, Download: Allow</t>
         </is>
       </c>
     </row>
@@ -695,7 +695,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Engineer:Read:Allow;Write:Deny;Delete:Deny;Download:Allow;Manager:Read:Allow;Write:Allow;Delete:Allow;Download:Allow;Everyone:Read:Allow;Write:Deny;Delete:Deny;Download:Deny</t>
+          <t>Engineer: Read: Allow, Write: Deny, Delete: Deny, Download: Allow; Manager: Read: Allow, Write: Allow, Delete: Allow, Download: Allow; Everyone: Read: Allow, Write: Deny, Delete: Deny, Download: Deny</t>
         </is>
       </c>
     </row>
@@ -717,7 +717,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Manager:Read:Allow;Write:Allow;Delete:Allow;Download:Allow;Everyone:Read:Allow;Write:Deny;Delete:Deny;Download:Deny</t>
+          <t>Manager: Read: Allow, Write: Allow, Delete: Allow, Download: Allow; Everyone: Read: Allow, Write: Deny, Delete: Deny, Download: Deny</t>
         </is>
       </c>
     </row>

</xml_diff>